<commit_message>
Roadmap: add 'New Ideas' sheet (icon interaction animations)
User-suggested backlog: settings cog rotate + static-icon pulse (quick win),
and the broader vision of bespoke in-character icon animations on tap, with a
feasibility note (draw-on/pop/pulse/rotate feasible now on the single-path
stroke icons; true shape-morphs like a hand closing need per-icon redesign).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Top 10 Visual" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Top 10 Wow" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Notes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="New Ideas" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +51,10 @@
       <color rgb="009C0006"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,6 +100,16 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1867,4 +1882,113 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>New Ideas (user-added backlog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Feasibility</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Detail / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Settings cog rotates on tap to match the nav-tab icon animation; static icons (e.g. chip) pulse</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Visual / Delight</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Feasible now — quick win</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Icons are single-path SVGs. Cog: add a rotate keyframe fired on click (the nav tabs already use a scale 'ad-tab-pop'). Pulse = scale/opacity loop. Low risk, ~1 small change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke, in-character icon animations on interaction — every icon reacts like the active nav-tab icon (e.g. lightning bolt shoots down, house constructs, book opens &amp; closes, hand closes, chip pulses)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Wow / Delight</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Partial — feasible subset now; full morphs are high-effort</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Feasible NOW on the existing single-path STROKE icons: stroke-dashoffset 'draw-on' (house 'constructs'), translate/fade (bolt 'shoots down'), rotate (cog), pulse (chip), pop. TRUE shape-morphs (a hand closing, a book opening/closing) can't be done on one static path — each needs redesigning as a multi-element / morphable SVG, or a Lottie-style asset (bigger design+eng project). Recommended path: ship cog + pulse + draw-on/pop first (covers most of the delight at low risk), tackle bespoke morphs icon-by-icon later.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Roadmap: mark icon tap-animations shipped (feasible tier)
Cog rotate + static-icon pulse = Done; bespoke in-character animations =
In Progress (transform-based tier shipped app-wide; true shape-morphs pending).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -1934,7 +1934,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="90" customHeight="1">
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Settings cog rotates on tap to match the nav-tab icon animation; static icons (e.g. chip) pulse</t>
@@ -1950,18 +1950,18 @@
           <t>Feasible now — quick win</t>
         </is>
       </c>
-      <c r="D3" s="11" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Icons are single-path SVGs. Cog: add a rotate keyframe fired on click (the nav tabs already use a scale 'ad-tab-pop'). Pulse = scale/opacity loop. Low risk, ~1 small change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="90" customHeight="1">
+          <t>Icons are single-path SVGs. Cog: add a rotate keyframe fired on click (the nav tabs already use a scale 'ad-tab-pop'). Pulse = scale/opacity loop. Low risk, ~1 small change.  [SHIPPED v2026.06.18.4: cog spins on tap; static icons (chip etc.) animate; delegated WAAPI listener covers every icon button.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Bespoke, in-character icon animations on interaction — every icon reacts like the active nav-tab icon (e.g. lightning bolt shoots down, house constructs, book opens &amp; closes, hand closes, chip pulses)</t>
@@ -1977,14 +1977,14 @@
           <t>Partial — feasible subset now; full morphs are high-effort</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Feasible NOW on the existing single-path STROKE icons: stroke-dashoffset 'draw-on' (house 'constructs'), translate/fade (bolt 'shoots down'), rotate (cog), pulse (chip), pop. TRUE shape-morphs (a hand closing, a book opening/closing) can't be done on one static path — each needs redesigning as a multi-element / morphable SVG, or a Lottie-style asset (bigger design+eng project). Recommended path: ship cog + pulse + draw-on/pop first (covers most of the delight at low risk), tackle bespoke morphs icon-by-icon later.</t>
+          <t>Feasible NOW on the existing single-path STROKE icons: stroke-dashoffset 'draw-on' (house 'constructs'), translate/fade (bolt 'shoots down'), rotate (cog), pulse (chip), pop. TRUE shape-morphs (a hand closing, a book opening/closing) can't be done on one static path — each needs redesigning as a multi-element / morphable SVG, or a Lottie-style asset (bigger design+eng project). Recommended path: ship cog + pulse + draw-on/pop first (covers most of the delight at low risk), tackle bespoke morphs icon-by-icon later.  [SHIPPED v2026.06.18.4 — feasible tier: spin/drop/build/swing/pulse/beat/pop mapped per icon, played on tap app-wide. REMAINING: true shape-morphs (hand closing, book opening) need per-icon SVG redesign.]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap log: add Bugs & Fixes sheet + post-audit Next-Up reprioritisation
Bugs & Fixes: logs the deploy-cache, Library/Browse overflow, and raised
bottom-nav issues (all fixed). Next-Up: my recommended order for remaining
work after the deep audit — configurator presets, CEFR validation and PWA
reminders rise; canvas/Browse polish falls; speaking stays the big bet;
tutor last.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -7,14 +7,16 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Top 10 Overall" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Top 10 UX" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Top 10 Learning" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Top 10 Retention" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Top 10 Visual" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Top 10 Wow" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Notes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="New Ideas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Bugs &amp; Fixes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Next-Up (post-audit)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Top 10 Overall" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Top 10 UX" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Top 10 Learning" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Top 10 Retention" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Top 10 Visual" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Top 10 Wow" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Notes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="New Ideas" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -24,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,6 +56,9 @@
     <font>
       <b val="1"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00006100"/>
     </font>
   </fonts>
   <fills count="4">
@@ -86,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -110,6 +115,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -477,211 +491,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Top 10 Overall</t>
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Bugs &amp; Fixes — session log</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Initiative</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Root cause</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Fix</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>2026.06.18.~</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Deploys not reaching devices ('nothing changed')</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Service-worker CACHE_NAME wasn't bumped (a manual, easily-missed deploy step), so installed PWAs kept the cached bundle.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>build now derives CACHE_NAME from a content hash of app.js+data.js+index.html — auto-invalidates every deploy.</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>2026.06.18.3</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Horizontal scroll in Library → word Browse on narrow phones; the 'Known' button overhung the card edge</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>CSS grid blow-out: grid tracks are auto-sized and items default to min-width:auto, so cards couldn't shrink below their content.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Grid -&gt; minmax(0,1fr); card minWidth:0; left column flex:1 + every text line ellipsised. Verified 280-390px.</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>2026.06.18.6</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Bottom tab bar raised up; dead gap (~1/8 screen) below it</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>The global overflow-x:hidden guard added in the fix above forced overflow-y:auto, turning the BODY into a scroll container; on mobile a fixed bottom bar then references the smaller layout viewport.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Removed the html/body overflow guard (overflow already prevented at source by the grid fixes). Body overflow-y back to 'visible'. Left a warning comment.</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="90" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>New Ideas (user-added backlog)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Idea</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Feasibility</t>
+        </is>
+      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Detail / done this session</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Re-rank progress to a moving metric</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Detail / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Settings cog rotates on tap to match the nav-tab icon animation; static icons (e.g. chip) pulse</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Visual / Delight</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>Feasible now — quick win</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Layered 'Strong' metric — journey %, rank, chapters now advance on SRS box&gt;=3 / 3-streak; Mastered * kept as deeper layer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Reviews Due as Home hero action</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Gold 'Review N due' hero on Home when reviews are due; new-session CTA demoted to outline (single focal point).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Compose the session canvas / remove void</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Icons are single-path SVGs. Cog: add a rotate keyframe fired on click (the nav tabs already use a scale 'ad-tab-pop'). Pulse = scale/opacity loop. Low risk, ~1 small change.  [SHIPPED v2026.06.18.4: cog spins on tap; static icons (chip etc.) animate; delegated WAAPI listener covers every icon button.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke, in-character icon animations on interaction — every icon reacts like the active nav-tab icon (e.g. lightning bolt shoots down, house constructs, book opens &amp; closes, hand closes, chip pulses)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Wow / Delight</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Partial — feasible subset now; full morphs are high-effort</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Answered state + recall card composed, example fills the void. MC-drill / typed-question void still to do.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Add production-output mode (writing/speaking)</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>5</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Redesign answered state into one calm verdict</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>One calm verdict block (SRS outcome + 5-dot mastery + quiet tutor link) replaces the 5-colour chip stack.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>6</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Replace Browse with curated discovery</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Aspirational empty states</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CEFR validation and truthful B2 progress</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Reposition around relocating professionals</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>10</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>AI Tutor productization (future premium launch feature)</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Feasible NOW on the existing single-path STROKE icons: stroke-dashoffset 'draw-on' (house 'constructs'), translate/fade (bolt 'shoots down'), rotate (cog), pulse (chip), pop. TRUE shape-morphs (a hand closing, a book opening/closing) can't be done on one static path — each needs redesigning as a multi-element / morphable SVG, or a Lottie-style asset (bigger design+eng project). Recommended path: ship cog + pulse + draw-on/pop first (covers most of the delight at low risk), tackle bespoke morphs icon-by-icon later.  [SHIPPED v2026.06.18.4 — feasible tier: spin/drop/build/swing/pulse/beat/pop mapped per icon, played on tap app-wide. REMAINING: true shape-morphs (hand closing, book opening) need per-icon SVG redesign.]</t>
         </is>
       </c>
     </row>
@@ -696,216 +736,343 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="74" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Top 10 UX</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>Next-Up — reprioritised after the deep audit (my recommendation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="46" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Order reflects what I learned actually building &amp; auditing the app: friction-cuts and data-integrity rise; canvas/Browse polish falls (worst parts already done, and typed-mode 'void' is keyboard space); speaking stays the big learning bet; tutor last (per direction).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Initiative</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Detail / done this session</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Why now (post-audit rationale)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="66" customHeight="1">
+      <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>One dominant Home action</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Single dominant gold action on Home (Due when due, else Production); other actions demoted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Configurator -&gt; 3 presets + Advanced</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Biggest friction-per-effort: the 5-axis setup modal gates EVERY session start and is shared by Home/Library/Train launches, so one change has broad reach. Pure layout.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Low-Med</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="66" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Surface SRS Due queue as daily anchor</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>SRS Due queue surfaced as the Home hero / daily anchor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Validate CEFR tags -&gt; truthful B2 %</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Audit found only ~1,000 of 2,001 words have a real CEFR level; the rest are guessed from difficulty (only 3 are tagged A1). The whole 'journey to B2 %' rests on this. Data task.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Med (data)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="66" customHeight="1">
+      <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Configurator → presets + Advanced</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>PWA reminders / re-engagement</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>The one retention lever still untouched. SRS apps live or die on the return trigger; 'you have N reviews due' as a notification is exactly the honest hook this app should own.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Low-Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Curated Browse experience</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Aspirational empty states</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Quick first-week 'aha': a brand-new user's Stats is a wall of zeros. Low effort, contained.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="66" customHeight="1">
+      <c r="A8" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Compose session canvas</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Recall card eyebrow + answered verdict composed; remaining session screens pending.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Personalised weak-spot deck</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Data already exists (per-card miss counts + the Weak queue). Turn it into a first-class 'drill your weak spots' deck. Real learning value, modest build.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1">
+      <c r="A9" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Redesign answered metadata stack</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Answered metadata stack redesigned into one verdict block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Speaking production mode</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>The biggest remaining LEARNING gap — B2 means speaking, and the app trains none. Web-Speech de-DE shadowing + scoring; speechSynthesis (output) already wired, recognition (input) is the new part.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="66" customHeight="1">
+      <c r="A10" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Remove redundant header eyebrows</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Finish session-canvas composition (MC/tap screens)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>DOWNGRADED. Worst offenders (answered state, recall card) already composed, and typed-mode 'void' is keyboard territory. Remaining: port the Audio bottom-anchor to the article/verb-MC/sentence screens.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="66" customHeight="1">
+      <c r="A11" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Progressive disclosure in Progress/Stats</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Curated Browse (grouping / sticky letters)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>DOWNGRADED. Overflow fixed and search works, so the flat list is usable; curation is now polish, not a pain point.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Unify naming and labels</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Relocation scenario packs + reposition</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Identity bet (the defensible niche). Content + copy heavy; sequence after the friction/retention wins land.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Med-High</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Listening-first mode</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Listening-first dialogues: German hidden ('Tap to listen') until heard; Read-along toggle, persisted.</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>AI-graded writing</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Pairs with the tutor; needs the hosted proxy. Real B2 'write to the Bürgeramt' value.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>AI Tutor productisation</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Deferred per your direction — the premium-tier capstone, do last. Needs metered hosted proxy.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Already shipped this session (for context):</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>Layered 'Strong' progress · Due-as-hero · one-verdict answered state · vocab-in-context · listening-first · faster chapters · grammar (modal/separable) fix · tap-driven icon animations + cog redesign · Library/Browse overflow + bottom-nav fixes · auto cache-bump deploys.</t>
         </is>
       </c>
     </row>
@@ -932,7 +1099,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Top 10 Learning</t>
+          <t>Top 10 Overall</t>
         </is>
       </c>
     </row>
@@ -964,7 +1131,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Layered mastery system</t>
+          <t>Re-rank progress to a moving metric</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -974,7 +1141,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Encountered -&gt; Learning -&gt; Strong -&gt; Mastered; public progress advances on Strong.</t>
+          <t>Layered 'Strong' metric — journey %, rank, chapters now advance on SRS box&gt;=3 / 3-streak; Mastered * kept as deeper layer.</t>
         </is>
       </c>
     </row>
@@ -984,12 +1151,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Speaking production mode</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Reviews Due as Home hero action</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Gold 'Review N due' hero on Home when reviews are due; new-session CTA demoted to outline (single focal point).</t>
         </is>
       </c>
     </row>
@@ -999,12 +1171,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AI-graded writing</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Compose the session canvas / remove void</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Answered state + recall card composed, example fills the void. MC-drill / typed-question void still to do.</t>
         </is>
       </c>
     </row>
@@ -1014,17 +1191,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Hand-author irregular/modal grammar rules</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>verbRule now flags present-irregular (modals, sein, wissen) + separable verbs; 'wollen -&gt; ich will' no longer mislabelled 'keeps its stem'.</t>
+          <t>Add production-output mode (writing/speaking)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1034,12 +1206,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Validate CEFR tags</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Redesign answered state into one calm verdict</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>One calm verdict block (SRS outcome + 5-dot mastery + quiet tutor link) replaces the 5-colour chip stack.</t>
         </is>
       </c>
     </row>
@@ -1049,17 +1226,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Vocabulary-in-context practice</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Example sentence shown by default in production answered state, target word highlighted (data already on all 2,001 cards).</t>
+          <t>Replace Browse with curated discovery</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1241,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Personalized weak-spot deck</t>
+          <t>Aspirational empty states</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1084,17 +1256,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Listening-first comprehension</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Listening-first comprehension in the 87 dialogues.</t>
+          <t>CEFR validation and truthful B2 progress</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1271,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Confusion-pair drilling</t>
+          <t>Reposition around relocating professionals</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1119,7 +1286,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Exam-format practice</t>
+          <t>AI Tutor productization (future premium launch feature)</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1151,7 +1318,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Top 10 Retention</t>
+          <t>Top 10 UX</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1350,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Moving progress metric</t>
+          <t>One dominant Home action</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1193,7 +1360,7 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Moving 'Strong' progress metric (was welded to 5-in-a-row mastery).</t>
+          <t>Single dominant gold action on Home (Due when due, else Production); other actions demoted.</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1370,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Reviews Due return trigger</t>
+          <t>Surface SRS Due queue as daily anchor</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1213,7 +1380,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Reviews Due as the Home hero return-trigger.</t>
+          <t>SRS Due queue surfaced as the Home hero / daily anchor.</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1390,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PWA reminders/notifications</t>
+          <t>Configurator → presets + Advanced</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -1238,7 +1405,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Competence-based milestones</t>
+          <t>Curated Browse experience</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1253,12 +1420,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Adaptive daily plan</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Compose session canvas</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Recall card eyebrow + answered verdict composed; remaining session screens pending.</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1440,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Weekly recap</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Redesign answered metadata stack</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Answered metadata stack redesigned into one verdict block.</t>
         </is>
       </c>
     </row>
@@ -1283,17 +1460,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Human progress language</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Headline copy now 'learned'/'solid' instead of 'mastered'; competence-based phrasing ('you can now...') still to come.</t>
+          <t>Remove redundant header eyebrows</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1475,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Streak-freeze visibility</t>
+          <t>Progressive disclosure in Progress/Stats</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1318,7 +1490,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>First-week aha sequence</t>
+          <t>Unify naming and labels</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1333,7 +1505,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Faster chapter progression</t>
+          <t>Listening-first mode</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1343,7 +1515,7 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Chapters fill on Strong, so a checkpoint / rank-up is reachable in days, not months.</t>
+          <t>Listening-first dialogues: German hidden ('Tap to listen') until heard; Read-along toggle, persisted.</t>
         </is>
       </c>
     </row>
@@ -1370,7 +1542,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Top 10 Visual</t>
+          <t>Top 10 Learning</t>
         </is>
       </c>
     </row>
@@ -1402,17 +1574,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Compose session canvas</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>Layered mastery system</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Recall card eyebrow + answered verdict + in-context example; MC/audio-style anchor for remaining screens pending.</t>
+          <t>Encountered -&gt; Learning -&gt; Strong -&gt; Mastered; public progress advances on Strong.</t>
         </is>
       </c>
     </row>
@@ -1422,17 +1594,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Screen-level focal point rule</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Home now has one gold focal action; not yet a systematic per-screen rule.</t>
+          <t>Speaking production mode</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1442,17 +1609,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Ration colour usage</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Answered state reduced to one accent colour; app-wide colour rationing pending.</t>
+          <t>AI-graded writing</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1624,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Redesign answered state</t>
+          <t>Hand-author irregular/modal grammar rules</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1472,7 +1634,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Answered state redesigned into one calm verdict.</t>
+          <t>verbRule now flags present-irregular (modals, sein, wissen) + separable verbs; 'wollen -&gt; ich will' no longer mislabelled 'keeps its stem'.</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1644,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Aspirational empty states</t>
+          <t>Validate CEFR tags</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1497,12 +1659,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Improve Sentence Builder visual language</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Vocabulary-in-context practice</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Example sentence shown by default in production answered state, target word highlighted (data already on all 2,001 cards).</t>
         </is>
       </c>
     </row>
@@ -1512,17 +1679,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Improve Home hierarchy</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>Home hierarchy: Due hero + demoted secondary CTAs; action now outranks the wordmark.</t>
+          <t>Personalized weak-spot deck</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1532,17 +1694,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tighten card spacing</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>Listening-first comprehension</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Recall card balanced with an eyebrow; single-line vertical-centering still present elsewhere.</t>
+          <t>Listening-first comprehension in the 87 dialogues.</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1714,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Remove duplicate progress indicators</t>
+          <t>Confusion-pair drilling</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1567,7 +1729,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Use Audio mode as composition benchmark</t>
+          <t>Exam-format practice</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1599,7 +1761,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Top 10 Wow</t>
+          <t>Top 10 Retention</t>
         </is>
       </c>
     </row>
@@ -1631,12 +1793,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Speaking with pronunciation scoring</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Moving progress metric</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Moving 'Strong' progress metric (was welded to 5-in-a-row mastery).</t>
         </is>
       </c>
     </row>
@@ -1646,12 +1813,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>AI-graded writing feedback</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Reviews Due return trigger</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Reviews Due as the Home hero return-trigger.</t>
         </is>
       </c>
     </row>
@@ -1661,17 +1833,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Alive/composed session canvas</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>Session canvas partially composed (answered state, recall card, in-context example); full 'alive' canvas pending.</t>
+          <t>PWA reminders/notifications</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
         </is>
       </c>
     </row>
@@ -1681,7 +1848,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Relocation scenario packs</t>
+          <t>Competence-based milestones</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1696,7 +1863,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Goethe/telc exam mode</t>
+          <t>Adaptive daily plan</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1711,7 +1878,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Adaptive coach-style daily plan</t>
+          <t>Weekly recap</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1726,12 +1893,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Competence unlocks</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Human progress language</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Headline copy now 'learned'/'solid' instead of 'mastered'; competence-based phrasing ('you can now...') still to come.</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1913,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enhanced mastery celebrations</t>
+          <t>Streak-freeze visibility</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1756,7 +1928,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Native-speed real-world audio</t>
+          <t>First-week aha sequence</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1771,12 +1943,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Shareable progress recap</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+          <t>Faster chapter progression</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Chapters fill on Strong, so a checkpoint / rank-up is reachable in days, not months.</t>
         </is>
       </c>
     </row>
@@ -1786,6 +1963,439 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Top 10 Visual</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Initiative</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Detail / done this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Compose session canvas</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Recall card eyebrow + answered verdict + in-context example; MC/audio-style anchor for remaining screens pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Screen-level focal point rule</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Home now has one gold focal action; not yet a systematic per-screen rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ration colour usage</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Answered state reduced to one accent colour; app-wide colour rationing pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Redesign answered state</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Answered state redesigned into one calm verdict.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Aspirational empty states</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Improve Sentence Builder visual language</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Improve Home hierarchy</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Home hierarchy: Due hero + demoted secondary CTAs; action now outranks the wordmark.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tighten card spacing</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Recall card balanced with an eyebrow; single-line vertical-centering still present elsewhere.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Remove duplicate progress indicators</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Use Audio mode as composition benchmark</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Top 10 Wow</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Initiative</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Detail / done this session</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Speaking with pronunciation scoring</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AI-graded writing feedback</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Alive/composed session canvas</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Session canvas partially composed (answered state, recall card, in-context example); full 'alive' canvas pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Relocation scenario packs</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Goethe/telc exam mode</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Adaptive coach-style daily plan</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Competence unlocks</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Enhanced mastery celebrations</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Native-speed real-world audio</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Shareable progress recap</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1882,113 +2492,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="9" t="inlineStr">
-        <is>
-          <t>New Ideas (user-added backlog)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Idea</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Feasibility</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Detail / notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="120" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Settings cog rotates on tap to match the nav-tab icon animation; static icons (e.g. chip) pulse</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Visual / Delight</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Feasible now — quick win</t>
-        </is>
-      </c>
-      <c r="D3" s="10" t="inlineStr">
-        <is>
-          <t>Done</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Icons are single-path SVGs. Cog: add a rotate keyframe fired on click (the nav tabs already use a scale 'ad-tab-pop'). Pulse = scale/opacity loop. Low risk, ~1 small change.  [SHIPPED v2026.06.18.4: cog spins on tap; static icons (chip etc.) animate; delegated WAAPI listener covers every icon button.]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="150" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Bespoke, in-character icon animations on interaction — every icon reacts like the active nav-tab icon (e.g. lightning bolt shoots down, house constructs, book opens &amp; closes, hand closes, chip pulses)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Wow / Delight</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Partial — feasible subset now; full morphs are high-effort</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Feasible NOW on the existing single-path STROKE icons: stroke-dashoffset 'draw-on' (house 'constructs'), translate/fade (bolt 'shoots down'), rotate (cog), pulse (chip), pop. TRUE shape-morphs (a hand closing, a book opening/closing) can't be done on one static path — each needs redesigning as a multi-element / morphable SVG, or a Lottie-style asset (bigger design+eng project). Recommended path: ship cog + pulse + draw-on/pop first (covers most of the delight at low risk), tackle bespoke morphs icon-by-icon later.  [SHIPPED v2026.06.18.4 — feasible tier: spin/drop/build/swing/pulse/beat/pop mapped per icon, played on tap app-wide. REMAINING: true shape-morphs (hand closing, book opening) need per-icon SVG redesign.]</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Roadmap: mark configurator presets shipped
Top 10 UX #3 -> Done; Next-Up #1 -> Done (next effective priority is CEFR
tag validation).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -788,20 +788,22 @@
       </c>
     </row>
     <row r="4" ht="66" customHeight="1">
-      <c r="A4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Configurator -&gt; 3 presets + Advanced</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Configurator -&gt; presets + Advanced  [DONE v2026.06.18.7]</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>Biggest friction-per-effort: the 5-axis setup modal gates EVERY session start and is shared by Home/Library/Train launches, so one change has broad reach. Pure layout.</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Low-Med</t>
         </is>
@@ -1062,6 +1064,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1072,7 +1075,7 @@
     <row r="17" ht="60" customHeight="1">
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Layered 'Strong' progress · Due-as-hero · one-verdict answered state · vocab-in-context · listening-first · faster chapters · grammar (modal/separable) fix · tap-driven icon animations + cog redesign · Library/Browse overflow + bottom-nav fixes · auto cache-bump deploys.</t>
+          <t>Layered 'Strong' progress · Due-as-hero · one-verdict answered state · vocab-in-context · listening-first · faster chapters · grammar (modal/separable) fix · tap-driven icon animations + cog redesign · Library/Browse overflow + bottom-nav fixes · auto cache-bump deploys · configurator presets + Advanced.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1387,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="60" customHeight="1">
       <c r="A5" t="n">
         <v>3</v>
       </c>
@@ -1393,9 +1396,14 @@
           <t>Configurator → presets + Advanced</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>SHIPPED v2026.06.18.7: topic setup leads with 3 one-tap presets (Quick/Standard/Deep); full controls behind 'Advanced options'. Special drills keep focused controls.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Curated word Browse: fix broken A–Z + add section headers
The Browse list sorted by w.de, so every der/die/das noun collapsed under "D"
("der Bahnhof", "die Straße", "das Auto" all filed together) — the alphabet was
meaningless. Now it sorts by the article-stripped word (der Bahnhof → "Bahnhof"
→ files under B), and the rows are grouped under sticky A–Z section headers for
rhythm and a sense of place. Cap raised 80→120.

Spreadsheet: marks "Curated Browse" Done (Overall #6, UX #4, Next-Up #8) and —
fixing earlier entries — applies the green "Done" fill the other AI uses to every
item I'd shipped (empty states, weak-spot deck, session-canvas), plus the green
Next-Up rows. All Top-10 "Done" status cells now verified green.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xvtrg8E9KghDpX6MYjAGtj
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -870,17 +870,17 @@
           <t xml:space="preserve">✓</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Aspirational empty states  [DONE v2026.06.18.8]</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Quick first-week 'aha': a brand-new user's Stats is a wall of zeros. Low effort, contained.</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -897,17 +897,17 @@
           <t xml:space="preserve">✓</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Personalised weak-spot deck  [DONE v2026.06.18.9]</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Data already exists (per-card miss counts + the Weak queue). Turn it into a first-class 'drill your weak spots' deck. Real learning value, modest build.</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -949,17 +949,17 @@
           <t xml:space="preserve">✓</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Finish session-canvas composition (MC/tap screens)  [DONE v2026.06.18.10]</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>DOWNGRADED. Worst offenders (answered state, recall card) already composed, and typed-mode 'void' is keyboard territory. Remaining: port the Audio bottom-anchor to the article/verb-MC/sentence screens.</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -971,20 +971,22 @@
       </c>
     </row>
     <row r="11" ht="66" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Curated Browse (grouping / sticky letters)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✓</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Curated Browse (grouping / sticky letters)  [DONE v2026.06.18.11]</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>DOWNGRADED. Overflow fixed and search works, so the flat list is usable; curation is now polish, not a pain point.</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
@@ -1183,7 +1185,7 @@
           <t>Compose the session canvas / remove void</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Done</t>
         </is>
@@ -1238,9 +1240,14 @@
           <t>Replace Browse with curated discovery</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
         </is>
       </c>
     </row>
@@ -1253,12 +1260,12 @@
           <t>Aspirational empty states</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Done</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Done v2026.06.18.8 — first-run Progress shows an aspirational preview (Journey roadmap + Your-progress-live panel + Start-your-first-session CTA) instead of all-zero panels.</t>
         </is>
@@ -1427,9 +1434,14 @@
           <t>Curated Browse experience</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
         </is>
       </c>
     </row>
@@ -1442,14 +1454,14 @@
           <t>Compose session canvas</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Done</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Recall card eyebrow + answered verdict composed; remaining session screens pending.</t>
+          <t xml:space="preserve">Done v2026.06.18.10 — MC/tap + answered screens composed as a centred group (no top-cluster/void); typed-unanswered stays top-anchored for the keyboard.</t>
         </is>
       </c>
     </row>
@@ -1701,12 +1713,12 @@
           <t>Personalized weak-spot deck</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Done</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">SHIPPED v2026.06.18.9: first-class Weak-spots deck on Home — promoted out of the cramped Today-s-work cell into its own card that previews the actual trouble words (most-missed first, e.g. der Kondensator / die Spannung) with a Drill-weak-spots CTA. Tap launches the existing Weak Areas session. Only shows when weak cards exist; secondary to the gold Due hero.</t>
         </is>
@@ -2039,7 +2051,7 @@
           <t>Compose session canvas</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Done</t>
         </is>
@@ -2119,12 +2131,12 @@
           <t>Aspirational empty states</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Done</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">SHIPPED v2026.06.18.8: brand-new Progress is no longer a wall of zeros — the B2 Journey roadmap leads, then a YOUR PROGRESS, LIVE panel previews Accuracy / Recall speed / Memory strength / Day streak with a Start your first session CTA. Gated on ds.attempts===0 so populated stats are unchanged.</t>
         </is>

</xml_diff>

<commit_message>
Roadmap: CEFR validation -> In Progress (A1 layer validated)
A1 cross-checked against the official telc A1.1/A1.2 wordlists (489 words
re-tagged, explicit coverage 50->71%). A2/B1 lists pending, so the item is
In Progress rather than Done.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -815,25 +815,27 @@
       </c>
     </row>
     <row r="5" ht="66" customHeight="1">
-      <c r="A5" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Validate CEFR tags -&gt; truthful B2 %</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>◑</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Validate CEFR tags -&gt; truthful B2 %  [A1 DONE v2026.06.18.12; A2/B1 lists pending]</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Audit found only ~1,000 of 2,001 words have a real CEFR level; the rest are guessed from difficulty (only 3 are tagged A1). The whole 'journey to B2 %' rests on this. Data task.</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
         <is>
           <t>Med (data)</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -867,12 +869,12 @@
     <row r="7" ht="66" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aspirational empty states  [DONE v2026.06.18.8]</t>
+          <t>Aspirational empty states  [DONE v2026.06.18.8]</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
@@ -894,12 +896,12 @@
     <row r="8" ht="66" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personalised weak-spot deck  [DONE v2026.06.18.9]</t>
+          <t>Personalised weak-spot deck  [DONE v2026.06.18.9]</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
@@ -946,12 +948,12 @@
     <row r="10" ht="66" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finish session-canvas composition (MC/tap screens)  [DONE v2026.06.18.10]</t>
+          <t>Finish session-canvas composition (MC/tap screens)  [DONE v2026.06.18.10]</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
@@ -973,12 +975,12 @@
     <row r="11" ht="66" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">✓</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Curated Browse (grouping / sticky letters)  [DONE v2026.06.18.11]</t>
+          <t>Curated Browse (grouping / sticky letters)  [DONE v2026.06.18.11]</t>
         </is>
       </c>
       <c r="C11" s="13" t="inlineStr">
@@ -1072,7 +1074,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" s="2" t="inlineStr">
         <is>
@@ -1187,12 +1188,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHIPPED v2026.06.18.10: composed the multiple-choice + tap screens (article / verb-MC / listening / sentence-builder) and every answered state — the prompt card + options now sit as one CENTERED group with balanced negative space instead of clustering at the top over a void. Typed-while-unanswered stays top-anchored (keyboard space). Card maxHeight:100%+overflowY guards the tall answered summaries. (Chose centred-group over pure bottom-anchor: keeps prompt and options together for read-then-answer scanning.)</t>
+          <t>SHIPPED v2026.06.18.10: composed the multiple-choice + tap screens (article / verb-MC / listening / sentence-builder) and every answered state — the prompt card + options now sit as one CENTERED group with balanced negative space instead of clustering at the top over a void. Typed-while-unanswered stays top-anchored (keyboard space). Card maxHeight:100%+overflowY guards the tall answered summaries. (Chose centred-group over pure bottom-anchor: keeps prompt and options together for read-then-answer scanning.)</t>
         </is>
       </c>
     </row>
@@ -1242,12 +1243,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
+          <t>SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
         </is>
       </c>
     </row>
@@ -1262,16 +1263,16 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done v2026.06.18.8 — first-run Progress shows an aspirational preview (Journey roadmap + Your-progress-live panel + Start-your-first-session CTA) instead of all-zero panels.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Done v2026.06.18.8 — first-run Progress shows an aspirational preview (Journey roadmap + Your-progress-live panel + Start-your-first-session CTA) instead of all-zero panels.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="110" customHeight="1">
       <c r="A10" t="n">
         <v>8</v>
       </c>
@@ -1280,9 +1281,14 @@
           <t>CEFR validation and truthful B2 progress</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>A1 LAYER VALIDATED v2026.06.18.12: cross-checked all 2,001 words vs the official telc 'Einfach gut!' A1.1+A1.2 wordlists (1,112 A1 lemmas). 489 confirmed A1 now carry explicit level:A1 (414 were heuristic, 74 fixed down from over-tagged A2/B1/B2). Explicit-level coverage 50%→71%; explicit A1 3→491. PENDING: A2/B1 lists (user providing); B2 has no single official list (frequency+review).</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1442,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
+          <t>SHIPPED v2026.06.18.11: curated the word Browse — fixed the broken A-Z (der/die/das nouns were all clustering under D; they now file under the noun letter, e.g. der Abend under A) and added sticky A-Z section headers for rhythm and a sense of place.</t>
         </is>
       </c>
     </row>
@@ -1456,12 +1462,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done v2026.06.18.10 — MC/tap + answered screens composed as a centred group (no top-cluster/void); typed-unanswered stays top-anchored for the keyboard.</t>
+          <t>Done v2026.06.18.10 — MC/tap + answered screens composed as a centred group (no top-cluster/void); typed-unanswered stays top-anchored for the keyboard.</t>
         </is>
       </c>
     </row>
@@ -1669,7 +1675,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="110" customHeight="1">
       <c r="A7" t="n">
         <v>5</v>
       </c>
@@ -1678,9 +1684,14 @@
           <t>Validate CEFR tags</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>A1 LAYER VALIDATED v2026.06.18.12: cross-checked all 2,001 words vs the official telc 'Einfach gut!' A1.1+A1.2 wordlists (1,112 A1 lemmas). 489 confirmed A1 now carry explicit level:A1 (414 were heuristic, 74 fixed down from over-tagged A2/B1/B2). Explicit-level coverage 50%→71%; explicit A1 3→491. PENDING: A2/B1 lists (user providing); B2 has no single official list (frequency+review).</t>
         </is>
       </c>
     </row>
@@ -1715,12 +1726,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHIPPED v2026.06.18.9: first-class Weak-spots deck on Home — promoted out of the cramped Today-s-work cell into its own card that previews the actual trouble words (most-missed first, e.g. der Kondensator / die Spannung) with a Drill-weak-spots CTA. Tap launches the existing Weak Areas session. Only shows when weak cards exist; secondary to the gold Due hero.</t>
+          <t>SHIPPED v2026.06.18.9: first-class Weak-spots deck on Home — promoted out of the cramped Today-s-work cell into its own card that previews the actual trouble words (most-missed first, e.g. der Kondensator / die Spannung) with a Drill-weak-spots CTA. Tap launches the existing Weak Areas session. Only shows when weak cards exist; secondary to the gold Due hero.</t>
         </is>
       </c>
     </row>
@@ -2053,12 +2064,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done v2026.06.18.10 — MC/tap + answered screens composed as a centred group (no top-cluster/void); typed-unanswered stays top-anchored for the keyboard.</t>
+          <t>Done v2026.06.18.10 — MC/tap + answered screens composed as a centred group (no top-cluster/void); typed-unanswered stays top-anchored for the keyboard.</t>
         </is>
       </c>
     </row>
@@ -2133,12 +2144,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Done</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">SHIPPED v2026.06.18.8: brand-new Progress is no longer a wall of zeros — the B2 Journey roadmap leads, then a YOUR PROGRESS, LIVE panel previews Accuracy / Recall speed / Memory strength / Day streak with a Start your first session CTA. Gated on ds.attempts===0 so populated stats are unchanged.</t>
+          <t>SHIPPED v2026.06.18.8: brand-new Progress is no longer a wall of zeros — the B2 Journey roadmap leads, then a YOUR PROGRESS, LIVE panel previews Accuracy / Recall speed / Memory strength / Day streak with a Start your first session CTA. Gated on ds.attempts===0 so populated stats are unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: CEFR A1-B1 validated for existing vocab (re-tag complete); add-new-words decision pending
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="66" customHeight="1">
+    <row r="5" ht="70" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>◑</t>
@@ -822,7 +822,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Validate CEFR tags -&gt; truthful B2 %  [A1 DONE v2026.06.18.12; A2/B1 lists pending]</t>
+          <t>Validate CEFR tags -&gt; truthful B2 %  [A1-B1 DONE v2026.06.18.13 for existing 2,001; pending: add ~2,236 new official words?, B2 list]</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -1272,7 +1272,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="110" customHeight="1">
+    <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
         <v>8</v>
       </c>
@@ -1288,7 +1288,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>A1 LAYER VALIDATED v2026.06.18.12: cross-checked all 2,001 words vs the official telc 'Einfach gut!' A1.1+A1.2 wordlists (1,112 A1 lemmas). 489 confirmed A1 now carry explicit level:A1 (414 were heuristic, 74 fixed down from over-tagged A2/B1/B2). Explicit-level coverage 50%→71%; explicit A1 3→491. PENDING: A2/B1 lists (user providing); B2 has no single official list (frequency+review).</t>
+          <t>A1-B1 VALIDATED for existing vocab v2026.06.18.13: all 2,001 words cross-checked vs the official telc A1.1-B1.2 wordlists (3,135 lemmas, clean table extraction). 889 words now authoritatively levelled (A1 492 / A2 247 / B1 150, A1 precedence); explicit coverage 50%-&gt;81%. REMAINING: (a) decide whether to ADD ~2,236 official words we don't have (would ~double the vocab), (b) B2 has no single official list (frequency+review).</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="110" customHeight="1">
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" t="n">
         <v>5</v>
       </c>
@@ -1691,7 +1691,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>A1 LAYER VALIDATED v2026.06.18.12: cross-checked all 2,001 words vs the official telc 'Einfach gut!' A1.1+A1.2 wordlists (1,112 A1 lemmas). 489 confirmed A1 now carry explicit level:A1 (414 were heuristic, 74 fixed down from over-tagged A2/B1/B2). Explicit-level coverage 50%→71%; explicit A1 3→491. PENDING: A2/B1 lists (user providing); B2 has no single official list (frequency+review).</t>
+          <t>A1-B1 VALIDATED for existing vocab v2026.06.18.13: all 2,001 words cross-checked vs the official telc A1.1-B1.2 wordlists (3,135 lemmas, clean table extraction). 889 words now authoritatively levelled (A1 492 / A2 247 / B1 150, A1 precedence); explicit coverage 50%-&gt;81%. REMAINING: (a) decide whether to ADD ~2,236 official words we don't have (would ~double the vocab), (b) B2 has no single official list (frequency+review).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: vocab-add batch 1 logged (+73 official A1 words)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -814,7 +814,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="84" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>◑</t>
@@ -822,7 +822,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Validate CEFR tags -&gt; truthful B2 %  [A1-B1 DONE v2026.06.18.13 for existing 2,001; pending: add ~2,236 new official words?, B2 list]</t>
+          <t>Validate CEFR + ADD official words. A1-B1 re-tag DONE (v.13). ADDING new official words w/ authored examples: 2,055 content words queued across 20 categories; BATCH 1 DONE v.14 (+73: Greetings/Family/Clothing). ~1,982 remaining, ~one category per batch.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -2453,10 +2453,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2541,6 +2541,27 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Official vocab add — progress</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Source: telc 'Einfach gut!' A1.1-B1.2. 2,055 new content words (function/multi-form filtered out), authored with example sentences, merged via scripts/merge_vocab.mjs into existing categories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Batch 1 (v2026.06.18.14): +73 — Greetings &amp; Basics 20, Family &amp; People 23, Clothing &amp; Style 30. Vocab 2,001 -&gt; 2,074.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: vocab-add batch 2 logged (+142; 215/~2,055 total)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -822,7 +822,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Validate CEFR + ADD official words. A1-B1 re-tag DONE (v.13). ADDING new official words w/ authored examples: 2,055 content words queued across 20 categories; BATCH 1 DONE v.14 (+73: Greetings/Family/Clothing). ~1,982 remaining, ~one category per batch.</t>
+          <t>Validate CEFR + ADD official words. A1-B1 re-tag DONE. ADDING (authored examples): 215 / ~2,055 done across batches 1-2 (build .15). ~1,840 remaining; ~one set of categories per batch, deployed each time.</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
@@ -2453,7 +2453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2562,6 +2562,13 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Batch 2 (v2026.06.18.15): +142 — Health &amp; Doctor 42, Body &amp; Health 60, Driving &amp; Traffic 40. Vocab 2,074 -&gt; 2,216. Running total added: 215 / ~2,055.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: vocab-add batch 3 logged (+101 Admin & Bureaucracy; 316/~2,055)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -26,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,6 +60,10 @@
     <font>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -91,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +130,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2453,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2569,6 +2574,13 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Batch 3 (v2026.06.19.01): +101 — Admin &amp; Bureaucracy 101. Relocation-critical Amt vocabulary (A2+B1). Running total added: 316/~2,055.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: vocab wave 1 logged (+662; 978/~2,055 total)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -2458,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2581,6 +2581,13 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Wave 1 (v2026.06.19.02): +662 across 27 categories — subagent-authored from telc A1-B1 lists (Food, Cooking, Shopping, Banking, Everyday Actions, Travel, etc.), each word re-categorised to the correct existing category with corrected glosses/articles/plurals. Vocab 2317-&gt;2979. Running total added: 978/~2,055.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: vocab waves 2-3 logged; official telc vocab add complete (2001->4013)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -2458,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2588,6 +2588,27 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Wave 2 (v2026.06.19.03): +1018 across 35 categories — subagent-authored (Housing, Work &amp; Study, Media, Engineering Workplace, Nature/Weather, Sport). Re-categorised + gloss/article/plural corrected. Vocab 2979-&gt;3997.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Wave 3 (v2026.06.19.04): +16 final stragglers (school subjects, die Tasse, der Plan, der Blick, niemand/irgendwer/irgendwelche). Vocab 3997-&gt;4013.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>OFFICIAL VOCAB ADD COMPLETE: ~2,012 new telc A1-B1 words added this session (batches 1-3 + waves 1-3). Vocab 2001 -&gt; 4013 across 36 categories. Function words, inflected forms, proper nouns and mis-glossed extraction artifacts were deliberately dropped. CEFR re-tag + official-list validation task closed out.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: log QA sweep + 100% CEFR coverage
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -2458,7 +2458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2609,6 +2609,20 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>QA sweep (post-add): heuristic check of all 2,012 new cards for cross-category duplicates, examples missing the headword, and suspicious glosses. 0 real defects — 91 flags were all false positives (separable verbs that split, umlaut plurals, and true cognates like fit/modern/beige). 0 cross-category duplicate words.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>CEFR coverage -&gt; 100% (v2026.06.19.05): tagged the remaining 374 legacy off-telc-list cards from their curated diff field using the deck-wide empirical mode (easy-&gt;A1, medium-&gt;A2, hard-&gt;B1). Final levels A1 1038 / A2 1307 / B1 1249 / B2 419, 0 untagged. CEFR task fully closed.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: mark CEFR + official-vocab-add initiative DONE
Flip Next-Up #5 from in-progress to done and refresh the Top-10 Overall /
Learning detail rows: deck 2,001 -> 4,013, 100% CEFR coverage.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -822,17 +822,17 @@
     <row r="5" ht="84" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>◑</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Validate CEFR + ADD official words. A1-B1 re-tag DONE. ADDING (authored examples): 215 / ~2,055 done across batches 1-2 (build .15). ~1,840 remaining; ~one set of categories per batch, deployed each time.</t>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Validate CEFR + ADD official words  [DONE v2026.06.19.05]</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>Audit found only ~1,000 of 2,001 words have a real CEFR level; the rest are guessed from difficulty (only 3 are tagged A1). The whole 'journey to B2 %' rests on this. Data task.</t>
+          <t>Audit found only ~1,000 of 2,001 words had a real CEFR level. RESOLVED: re-tagged vs telc lists, added ~2,012 official A1-B1 words (deck 2,001-&gt;4,013), and filled all remaining cards -&gt; 100% level coverage (A1 1038 / A2 1307 / B1 1249 / B2 419).</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CEFR validation and truthful B2 progress</t>
+          <t>CEFR validation and truthful B2 progress  [DONE v2026.06.19.05]</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -1293,7 +1293,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>A1-B1 VALIDATED for existing vocab v2026.06.18.13: all 2,001 words cross-checked vs the official telc A1.1-B1.2 wordlists (3,135 lemmas, clean table extraction). 889 words now authoritatively levelled (A1 492 / A2 247 / B1 150, A1 precedence); explicit coverage 50%-&gt;81%. REMAINING: (a) decide whether to ADD ~2,236 official words we don't have (would ~double the vocab), (b) B2 has no single official list (frequency+review).</t>
+          <t>DONE v2026.06.19.05. A1-B1 re-validated vs official telc lists; +2,012 official words added (2,001-&gt;4,013); 100% explicit CEFR coverage (A1 1038 / A2 1307 / B1 1249 / B2 419).</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Validate CEFR tags</t>
+          <t>Validate CEFR tags  [DONE v2026.06.19.05]</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>A1-B1 VALIDATED for existing vocab v2026.06.18.13: all 2,001 words cross-checked vs the official telc A1.1-B1.2 wordlists (3,135 lemmas, clean table extraction). 889 words now authoritatively levelled (A1 492 / A2 247 / B1 150, A1 precedence); explicit coverage 50%-&gt;81%. REMAINING: (a) decide whether to ADD ~2,236 official words we don't have (would ~double the vocab), (b) B2 has no single official list (frequency+review).</t>
+          <t>DONE v2026.06.19.05. A1-B1 re-validated vs official telc lists; +2,012 official words added (2,001-&gt;4,013); 100% explicit CEFR coverage.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: register 'Add Aspekte neu B2 vocab' as in-progress (Next-Up)
New source supplied by Jack. ~1,890 B2 words to be authored via the wave
pipeline. Marked in-progress so the parallel agent sees the active work.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -741,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -847,54 +847,54 @@
       </c>
     </row>
     <row r="6" ht="66" customHeight="1">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>◑</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>ADD Aspekte neu B2 vocabulary (full grind)</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>New source supplied by Jack (Aspekte neu B2 Kapitelwortschatz PDF, 10 chapters, no English). ~1,890 new B2 words being authored (translate + categorise + examples) via the same wave/subagent pipeline. Grows deck 4,013 -&gt; ~5,900, ~5x B2 content. IN PROGRESS.</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>High (data)</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Low-Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="66" customHeight="1">
+      <c r="A7" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>PWA reminders / re-engagement</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>The one retention lever still untouched. SRS apps live or die on the return trigger; 'you have N reviews due' as a notification is exactly the honest hook this app should own.</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Low-Med</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="66" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Aspirational empty states  [DONE v2026.06.18.8]</t>
-        </is>
-      </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Quick first-week 'aha': a brand-new user's Stats is a wall of zeros. Low effort, contained.</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
@@ -906,74 +906,74 @@
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
+          <t>Aspirational empty states  [DONE v2026.06.18.8]</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Quick first-week 'aha': a brand-new user's Stats is a wall of zeros. Low effort, contained.</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="66" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
           <t>Personalised weak-spot deck  [DONE v2026.06.18.9]</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Data already exists (per-card miss counts + the Weak queue). Turn it into a first-class 'drill your weak spots' deck. Real learning value, modest build.</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="66" customHeight="1">
-      <c r="A9" s="4" t="n">
+    <row r="10" ht="66" customHeight="1">
+      <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Speaking production mode</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>The biggest remaining LEARNING gap — B2 means speaking, and the app trains none. Web-Speech de-DE shadowing + scoring; speechSynthesis (output) already wired, recognition (input) is the new part.</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Med</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="66" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Finish session-canvas composition (MC/tap screens)  [DONE v2026.06.18.10]</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>DOWNGRADED. Worst offenders (answered state, recall card) already composed, and typed-mode 'void' is keyboard territory. Remaining: port the Audio bottom-anchor to the article/verb-MC/sentence screens.</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Med</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
         </is>
       </c>
     </row>
@@ -985,67 +985,69 @@
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
+          <t>Finish session-canvas composition (MC/tap screens)  [DONE v2026.06.18.10]</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>DOWNGRADED. Worst offenders (answered state, recall card) already composed, and typed-mode 'void' is keyboard territory. Remaining: port the Audio bottom-anchor to the article/verb-MC/sentence screens.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
           <t>Curated Browse (grouping / sticky letters)  [DONE v2026.06.18.11]</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>DOWNGRADED. Overflow fixed and search works, so the flat list is usable; curation is now polish, not a pain point.</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="66" customHeight="1">
-      <c r="A12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Relocation scenario packs + reposition</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Identity bet (the defensible niche). Content + copy heavy; sequence after the friction/retention wins land.</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Med-High</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Med</t>
         </is>
       </c>
     </row>
     <row r="13" ht="66" customHeight="1">
       <c r="A13" s="4" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>AI-graded writing</t>
+          <t>Relocation scenario packs + reposition</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Pairs with the tutor; needs the hosted proxy. Real B2 'write to the Bürgeramt' value.</t>
+          <t>Identity bet (the defensible niche). Content + copy heavy; sequence after the friction/retention wins land.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Med-High</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
@@ -1056,38 +1058,64 @@
     </row>
     <row r="14" ht="66" customHeight="1">
       <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>AI-graded writing</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Pairs with the tutor; needs the hosted proxy. Real B2 'write to the Bürgeramt' value.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Med</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>AI Tutor productisation</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Deferred per your direction — the premium-tier capstone, do last. Needs metered hosted proxy.</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E15" s="14" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="2" t="inlineStr">
+    <row r="16"/>
+    <row r="17" ht="60" customHeight="1">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Already shipped this session (for context):</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="B17" s="15" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Layered 'Strong' progress · Due-as-hero · one-verdict answered state · vocab-in-context · listening-first · faster chapters · grammar (modal/separable) fix · tap-driven icon animations + cog redesign · Library/Browse overflow + bottom-nav fixes · auto cache-bump deploys · configurator presets + Advanced.</t>
         </is>

</xml_diff>

<commit_message>
Roadmap: B2 add wave A logged (+591; 591/~1,905 in progress)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -859,7 +859,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>New source supplied by Jack (Aspekte neu B2 Kapitelwortschatz PDF, 10 chapters, no English). ~1,890 new B2 words being authored (translate + categorise + examples) via the same wave/subagent pipeline. Grows deck 4,013 -&gt; ~5,900, ~5x B2 content. IN PROGRESS.</t>
+          <t>New source supplied by Jack (Aspekte neu B2 Kapitelwortschatz, 10 chapters, no English). Translating + categorising + authoring B2 examples via the wave/subagent pipeline. IN PROGRESS: 591/~1,905 added (wave A: ch 1-3,6). Deck 4,013 -&gt; ~5,900 when complete.</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -1106,7 +1106,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="60" customHeight="1">
       <c r="B17" s="2" t="inlineStr">
         <is>
@@ -2486,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2651,6 +2650,13 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>B2 add — Aspekte neu (source: Jack, no English). Wave A (v2026.06.19.06): +591, chapters 1-3 + 6 (Heimat, Sprache, Arbeit &amp; Beruf, Gesundheit). Translated + categorised + B2 examples via subagents. Vocab 4013-&gt;4604. B2 progress: 591/~1,905.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: B2 add wave B logged (+601; 1,192/~1,905 in progress)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -859,7 +859,7 @@
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>New source supplied by Jack (Aspekte neu B2 Kapitelwortschatz, 10 chapters, no English). Translating + categorising + authoring B2 examples via the wave/subagent pipeline. IN PROGRESS: 591/~1,905 added (wave A: ch 1-3,6). Deck 4,013 -&gt; ~5,900 when complete.</t>
+          <t>New source (Aspekte neu B2, no English). Translating+categorising+B2 examples via wave pipeline. IN PROGRESS: 1,192/~1,905 (waves A+B: ch 1-6,8). Deck -&gt; ~5,900 when done.</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -2485,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2657,6 +2657,13 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>B2 add wave B (v2026.06.19.07): +601, chapters 4,5,8 (Zusammen leben, Wissenschaft, Geschichte). Vocab 4604-&gt;5205. B2 progress: 1,192/~1,905.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: mark Aspekte neu B2 add DONE; log waves A & C + completion
All 10 chapters added (+1,785 B2 words, deck 4,013 -> 5,782). Next-Up #6
flipped to done. B2-level content 419 -> 2,167; 100% CEFR coverage held.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -849,17 +849,17 @@
     <row r="6" ht="66" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>◑</t>
+          <t>✓</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>ADD Aspekte neu B2 vocabulary (full grind)</t>
+          <t>ADD Aspekte neu B2 vocabulary  [DONE v2026.06.19.08]</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
         <is>
-          <t>New source (Aspekte neu B2, no English). Translating+categorising+B2 examples via wave pipeline. IN PROGRESS: 1,192/~1,905 (waves A+B: ch 1-6,8). Deck -&gt; ~5,900 when done.</t>
+          <t>Source supplied by Jack (Aspekte neu B2 Kapitelwortschatz, 10 chapters, no English). DONE: all 10 chapters translated+categorised+exemplified via the wave pipeline; +1,785 B2 words (deck 4,013 -&gt; 5,782). B2-level content 419 -&gt; 2,167. QA sweep clean; 100% CEFR coverage held.</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -2485,7 +2485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2664,6 +2664,27 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>B2 add wave A (v2026.06.19.07 prep / b0373cc): +591, chapters 1-3,6 (Heimat, Sprache, Arbeit, Gesundheit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>B2 add wave C (v2026.06.19.08): +577, chapters 7,9,10 (Kultur, Gefuehle, Zukunft). Repaired 3 cards truncated by an agent session-limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>ASPEKTE NEU B2 ADD COMPLETE (v2026.06.19.08): all 10 chapters added, +1,785 B2 words (deck 4,013 -&gt; 5,782). Translated from a German-only source via subagents (translate+categorise+author B2 examples from source collocations), consolidated to canonical categories, deduped, validated (26/26 tests). B2-level content 419 -&gt; 2,167. QA sweep clean (0 real defects), 100% CEFR coverage maintained. Levels: A1 1038 / A2 1307 / B1 1270 / B2 2167.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: reconcile status colours + notes across all sheets
- Next-Up #5 (CEFR) and #6 (B2): fill the whole row green to match the
  Done convention (C/D/E were left yellow).
- Top-10 Overall #10 and Top-10 Learning #7: flip status cell to green
  'Done' (was amber 'In Progress'); move status out of the initiative name.
- Notes: restyle appended rows to the body font; clean and chronologically
  order the B2 sub-section (Wave A/B/C + completion summary).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -830,17 +830,17 @@
           <t>Validate CEFR + ADD official words  [DONE v2026.06.19.05]</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>Audit found only ~1,000 of 2,001 words had a real CEFR level. RESOLVED: re-tagged vs telc lists, added ~2,012 official A1-B1 words (deck 2,001-&gt;4,013), and filled all remaining cards -&gt; 100% level coverage (A1 1038 / A2 1307 / B1 1249 / B2 419).</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Med (data)</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -857,17 +857,17 @@
           <t>ADD Aspekte neu B2 vocabulary  [DONE v2026.06.19.08]</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Source supplied by Jack (Aspekte neu B2 Kapitelwortschatz, 10 chapters, no English). DONE: all 10 chapters translated+categorised+exemplified via the wave pipeline; +1,785 B2 words (deck 4,013 -&gt; 5,782). B2-level content 419 -&gt; 2,167. QA sweep clean; 100% CEFR coverage held.</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>High (data)</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Low-Med</t>
         </is>
@@ -1310,17 +1310,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CEFR validation and truthful B2 progress  [DONE v2026.06.19.05]</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>CEFR validation and truthful B2 progress</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>DONE v2026.06.19.05. A1-B1 re-validated vs official telc lists; +2,012 official words added (2,001-&gt;4,013); 100% explicit CEFR coverage (A1 1038 / A2 1307 / B1 1249 / B2 419).</t>
+          <t>DONE v2026.06.19.08. A1-B1 re-validated vs official telc lists; +2,012 telc words then +1,785 Aspekte-neu B2 words (deck 2,001 -&gt; 5,782); 100% explicit CEFR coverage (A1 1038 / A2 1307 / B1 1270 / B2 2167).</t>
         </is>
       </c>
     </row>
@@ -1713,17 +1713,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Validate CEFR tags  [DONE v2026.06.19.05]</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>In Progress</t>
+          <t>Validate CEFR tags</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>DONE v2026.06.19.05. A1-B1 re-validated vs official telc lists; +2,012 official words added (2,001-&gt;4,013); 100% explicit CEFR coverage.</t>
+          <t>DONE v2026.06.19.08. A1-B1 re-validated vs telc lists; +2,012 telc + +1,785 Aspekte B2 words; 100% CEFR coverage; B2-level content 419 -&gt; 2,167.</t>
         </is>
       </c>
     </row>
@@ -2602,86 +2602,86 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Batch 3 (v2026.06.19.01): +101 — Admin &amp; Bureaucracy 101. Relocation-critical Amt vocabulary (A2+B1). Running total added: 316/~2,055.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Wave 1 (v2026.06.19.02): +662 across 27 categories — subagent-authored from telc A1-B1 lists (Food, Cooking, Shopping, Banking, Everyday Actions, Travel, etc.), each word re-categorised to the correct existing category with corrected glosses/articles/plurals. Vocab 2317-&gt;2979. Running total added: 978/~2,055.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Wave 2 (v2026.06.19.03): +1018 across 35 categories — subagent-authored (Housing, Work &amp; Study, Media, Engineering Workplace, Nature/Weather, Sport). Re-categorised + gloss/article/plural corrected. Vocab 2979-&gt;3997.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>Wave 3 (v2026.06.19.04): +16 final stragglers (school subjects, die Tasse, der Plan, der Blick, niemand/irgendwer/irgendwelche). Vocab 3997-&gt;4013.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>OFFICIAL VOCAB ADD COMPLETE: ~2,012 new telc A1-B1 words added this session (batches 1-3 + waves 1-3). Vocab 2001 -&gt; 4013 across 36 categories. Function words, inflected forms, proper nouns and mis-glossed extraction artifacts were deliberately dropped. CEFR re-tag + official-list validation task closed out.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>QA sweep (post-add): heuristic check of all 2,012 new cards for cross-category duplicates, examples missing the headword, and suspicious glosses. 0 real defects — 91 flags were all false positives (separable verbs that split, umlaut plurals, and true cognates like fit/modern/beige). 0 cross-category duplicate words.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>CEFR coverage -&gt; 100% (v2026.06.19.05): tagged the remaining 374 legacy off-telc-list cards from their curated diff field using the deck-wide empirical mode (easy-&gt;A1, medium-&gt;A2, hard-&gt;B1). Final levels A1 1038 / A2 1307 / B1 1249 / B2 419, 0 untagged. CEFR task fully closed.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>B2 add — Aspekte neu (source: Jack, no English). Wave A (v2026.06.19.06): +591, chapters 1-3 + 6 (Heimat, Sprache, Arbeit &amp; Beruf, Gesundheit). Translated + categorised + B2 examples via subagents. Vocab 4013-&gt;4604. B2 progress: 591/~1,905.</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>B2 add — Aspekte neu B2 (source: Jack; German-only PDF, 10 chapters, no English):</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>B2 add wave B (v2026.06.19.07): +601, chapters 4,5,8 (Zusammen leben, Wissenschaft, Geschichte). Vocab 4604-&gt;5205. B2 progress: 1,192/~1,905.</t>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Wave A (b0373cc, v2026.06.19.07): +591 — chapters 1-3,6 (Heimat, Sprache, Arbeit, Gesundheit).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
-        <is>
-          <t>B2 add wave A (v2026.06.19.07 prep / b0373cc): +591, chapters 1-3,6 (Heimat, Sprache, Arbeit, Gesundheit).</t>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Wave B (v2026.06.19.07): +601 — chapters 4,5,8 (Zusammen leben, Wissenschaft, Geschichte).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>B2 add wave C (v2026.06.19.08): +577, chapters 7,9,10 (Kultur, Gefuehle, Zukunft). Repaired 3 cards truncated by an agent session-limit.</t>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Wave C (v2026.06.19.08): +577 — chapters 7,9,10 (Kultur, Gefuehle, Zukunft). Repaired 3 cards truncated by an agent session-limit.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
-        <is>
-          <t>ASPEKTE NEU B2 ADD COMPLETE (v2026.06.19.08): all 10 chapters added, +1,785 B2 words (deck 4,013 -&gt; 5,782). Translated from a German-only source via subagents (translate+categorise+author B2 examples from source collocations), consolidated to canonical categories, deduped, validated (26/26 tests). B2-level content 419 -&gt; 2,167. QA sweep clean (0 real defects), 100% CEFR coverage maintained. Levels: A1 1038 / A2 1307 / B1 1270 / B2 2167.</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ASPEKTE NEU B2 ADD COMPLETE (v2026.06.19.08): +1,785 B2 words via subagents (translate+categorise+author B2 examples from source collocations), consolidated to canonical categories, deduped, validated (26/26 tests). Deck 4,013 -&gt; 5,782. B2-level content 419 -&gt; 2,167. QA sweep clean. 100% CEFR coverage held: A1 1038 / A2 1307 / B1 1270 / B2 2167.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Roadmap: mark PWA daily reminders DONE (Next-Up #3, Retention #5)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -874,25 +874,27 @@
       </c>
     </row>
     <row r="7" ht="66" customHeight="1">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>PWA reminders / re-engagement</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>The one retention lever still untouched. SRS apps live or die on the return trigger; 'you have N reviews due' as a notification is exactly the honest hook this app should own.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>PWA reminders / re-engagement  [DONE v2026.06.19.09]</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Shipped: opt-in Daily Reminder (Settings) — local notification at a chosen time, skips days the goal is met. Notification Triggers API where available (fires when closed), foreground-timer fallback. No backend. iOS reminds best while the app is opened periodically.</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Low-Med</t>
         </is>
@@ -1915,9 +1917,14 @@
           <t>PWA reminders/notifications</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Not Started</t>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Done v2026.06.19.09 — opt-in daily reminder: Settings toggle + time picker, gentle local notification that defends the streak and skips days the goal is already met. Notification Triggers API when available (fires while closed), foreground fallback otherwise; no backend.</t>
         </is>
       </c>
     </row>
@@ -2485,7 +2492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -2685,6 +2692,13 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Daily reminder shipped (v2026.06.19.09): opt-in Settings toggle + time picker; gentle local notification to defend the streak, skipped when the day’s goal is met. Uses the Notification Triggers API where available (fires when the app is closed; re-armed on open) with a foreground-timer fallback; SW notificationclick focuses/opens the app. No backend. Closes Next-Up #3 / Retention #5.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Roadmap: log level-aware sessions regression fix (Bugs & Fixes)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LN6TW75L2UGFxYaYn7Ggia
</commit_message>
<xml_diff>
--- a/AutoDeutsch_Roadmap_Checklist.xlsx
+++ b/AutoDeutsch_Roadmap_Checklist.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -616,6 +616,33 @@
         </is>
       </c>
       <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026.06.19.10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Beginners swamped with B2 vocab; level preference silently reset</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>After the deck grew to 5,782 words (37% B2), the default session level was the flat "all" pool, and the one-tap presets (Quick/Standard/Deep) hardcoded level:"all" and persisted it — overwriting the learner's level and pulling B2 words into A1 sessions.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>setupLevel now defaults to "auto" (resolved to the learner's current CEFR level in filterPool, auto-advancing A1→A2→B1→B2); presets honour the level filter instead of forcing/persisting "all"; added an "Auto" selector option + hint; one-time migration of the legacy "all" default to "auto" (explicit bands kept). Fresh all-categories pool: 1,038 A1 cards, not 5,782 mixed.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>